<commit_message>
updates based on tests with recent data
</commit_message>
<xml_diff>
--- a/stats.xlsx
+++ b/stats.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\brice\Desktop\Projects\LIBRA-II\Software\SfM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C86443F5-3DDB-4123-BB88-7C4B85699047}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC1801E6-05C3-4F5D-9D39-FB9BBF0A9A3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B23DA20A-2892-4B18-A9C1-EE055436BAD8}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Main" sheetId="1" r:id="rId1"/>
+    <sheet name="Visualization" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="26">
   <si>
     <t>Camera</t>
   </si>
@@ -81,13 +82,47 @@
   </si>
   <si>
     <t>Total</t>
+  </si>
+  <si>
+    <t>Exhaustive</t>
+  </si>
+  <si>
+    <t>Sequential</t>
+  </si>
+  <si>
+    <t>VocabTree</t>
+  </si>
+  <si>
+    <t>Spatial</t>
+  </si>
+  <si>
+    <t>Transitive</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>2024-1-24_Captures-for-SfM\with-flashlight\a_Y-only\0_project.ini</t>
+  </si>
+  <si>
+    <t>2024-1-24_Captures-for-SfM\no-flashlight\c_X-and-Y\project.ini</t>
+  </si>
+  <si>
+    <t>2024-1-24_Captures-for-SfM\no-flashlight\b_X-only\project.ini</t>
+  </si>
+  <si>
+    <t>2024-1-24_Captures-for-SfM\no-flashlight\a_Y-only\project.ini</t>
+  </si>
+  <si>
+    <t>2024-1-24_Captures-for-SfM\with-flashlight\a_Y-only\?_project.ini</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
@@ -204,44 +239,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -304,6 +306,46 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -619,395 +661,657 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11E653C8-A8C7-445C-A865-F01C0238B771}">
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:Q22"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" zeroHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.140625" style="35" customWidth="1"/>
-    <col min="2" max="2" width="8.5703125" style="32" customWidth="1"/>
-    <col min="3" max="3" width="12.85546875" style="29" customWidth="1"/>
-    <col min="4" max="4" width="12.85546875" style="2" customWidth="1"/>
-    <col min="5" max="6" width="12.85546875" style="1" customWidth="1"/>
-    <col min="7" max="10" width="10" style="1" customWidth="1"/>
-    <col min="11" max="11" width="10" style="3" customWidth="1"/>
-    <col min="12" max="12" width="12.85546875" style="15" customWidth="1"/>
-    <col min="13" max="16384" width="9.140625" hidden="1"/>
+    <col min="1" max="1" width="22.85546875" style="24" customWidth="1"/>
+    <col min="2" max="2" width="8.5703125" style="21" customWidth="1"/>
+    <col min="3" max="3" width="12.85546875" style="18" customWidth="1"/>
+    <col min="4" max="4" width="12.85546875" style="32" customWidth="1"/>
+    <col min="5" max="10" width="12.85546875" style="33" customWidth="1"/>
+    <col min="11" max="14" width="10" style="33" customWidth="1"/>
+    <col min="15" max="15" width="10" style="34" customWidth="1"/>
+    <col min="16" max="16" width="12.85546875" style="4" customWidth="1"/>
+    <col min="17" max="17" width="64.28515625" style="36" customWidth="1"/>
+    <col min="18" max="16384" width="9.140625" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="24" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+    <row r="1" spans="1:17" s="13" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="19" t="s">
+      <c r="D1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="21" t="s">
+      <c r="K1" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="23" t="s">
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="11"/>
+      <c r="P1" s="12" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" s="24" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16"/>
-      <c r="B2" s="17"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="25" t="s">
+      <c r="Q1" s="35" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" s="13" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="5"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="J2" s="9"/>
+      <c r="K2" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="25" t="s">
+      <c r="L2" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="25" t="s">
+      <c r="M2" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="25" t="s">
+      <c r="N2" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="K2" s="26" t="s">
+      <c r="O2" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="L2" s="23"/>
-    </row>
-    <row r="3" spans="1:12" s="7" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="33" t="s">
+      <c r="P2" s="12"/>
+      <c r="Q2" s="35"/>
+    </row>
+    <row r="3" spans="1:17" s="1" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="30">
+      <c r="B3" s="19">
         <v>45</v>
       </c>
-      <c r="C3" s="27" t="s">
+      <c r="C3" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="26">
         <v>2.1999999999999999E-2</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="27">
         <v>0.03</v>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="27"/>
+      <c r="G3" s="27"/>
+      <c r="H3" s="27"/>
+      <c r="I3" s="27"/>
+      <c r="J3" s="27">
         <v>0.222</v>
       </c>
-      <c r="G3" s="5">
+      <c r="K3" s="27">
         <v>1E-3</v>
       </c>
-      <c r="H3" s="5">
+      <c r="L3" s="27">
         <v>15.677</v>
       </c>
-      <c r="I3" s="5">
+      <c r="M3" s="27">
         <v>0.2</v>
       </c>
-      <c r="J3" s="5">
+      <c r="N3" s="27">
         <v>0.29099999999999998</v>
       </c>
-      <c r="K3" s="6">
-        <v>8.8999999999999996E-2</v>
-      </c>
-      <c r="L3" s="12" t="str">
-        <f>TEXT(SUM(D3:K3)/1440,"hh:mm:ss")</f>
+      <c r="O3" s="28">
+        <v>8.8900000000000007E-2</v>
+      </c>
+      <c r="P3" s="3" t="str">
+        <f>TEXT(SUM(D3:O3)/1440,"hh:mm:ss")</f>
         <v>00:16:32</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" s="11" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="34"/>
-      <c r="B4" s="31">
+      <c r="Q3" s="37" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" s="2" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="20">
         <v>45</v>
       </c>
-      <c r="C4" s="28" t="s">
+      <c r="C4" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="8"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="10"/>
-      <c r="L4" s="13"/>
-    </row>
-    <row r="5" spans="1:12" s="7" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="33"/>
-      <c r="B5" s="30"/>
-      <c r="C5" s="27"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="6"/>
-      <c r="L5" s="14"/>
-    </row>
-    <row r="6" spans="1:12" s="11" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="34"/>
-      <c r="B6" s="31"/>
-      <c r="C6" s="28"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="10"/>
-      <c r="L6" s="13"/>
-    </row>
-    <row r="7" spans="1:12" s="7" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="33"/>
-      <c r="B7" s="30"/>
-      <c r="C7" s="27"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="14"/>
-    </row>
-    <row r="8" spans="1:12" s="11" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="34"/>
-      <c r="B8" s="31"/>
-      <c r="C8" s="28"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="10"/>
-      <c r="L8" s="13"/>
-    </row>
-    <row r="9" spans="1:12" s="7" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="33"/>
-      <c r="B9" s="30"/>
-      <c r="C9" s="27"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="6"/>
-      <c r="L9" s="14"/>
-    </row>
-    <row r="10" spans="1:12" s="11" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="34"/>
-      <c r="B10" s="31"/>
-      <c r="C10" s="28"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
-      <c r="K10" s="10"/>
-      <c r="L10" s="13"/>
-    </row>
-    <row r="11" spans="1:12" s="7" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="33"/>
-      <c r="B11" s="30"/>
-      <c r="C11" s="27"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="14"/>
-    </row>
-    <row r="12" spans="1:12" s="11" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="34"/>
-      <c r="B12" s="31"/>
-      <c r="C12" s="28"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="10"/>
-      <c r="L12" s="13"/>
-    </row>
-    <row r="13" spans="1:12" s="7" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="33"/>
-      <c r="B13" s="30"/>
-      <c r="C13" s="27"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="6"/>
-      <c r="L13" s="14"/>
-    </row>
-    <row r="14" spans="1:12" s="11" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="34"/>
-      <c r="B14" s="31"/>
-      <c r="C14" s="28"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
-      <c r="K14" s="10"/>
-      <c r="L14" s="13"/>
-    </row>
-    <row r="15" spans="1:12" s="7" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="33"/>
-      <c r="B15" s="30"/>
-      <c r="C15" s="27"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
-      <c r="K15" s="6"/>
-      <c r="L15" s="14"/>
-    </row>
-    <row r="16" spans="1:12" s="11" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="34"/>
-      <c r="B16" s="31"/>
-      <c r="C16" s="28"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="9"/>
-      <c r="J16" s="9"/>
-      <c r="K16" s="10"/>
-      <c r="L16" s="13"/>
-    </row>
-    <row r="17" spans="1:12" s="7" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="33"/>
-      <c r="B17" s="30"/>
-      <c r="C17" s="27"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5"/>
-      <c r="K17" s="6"/>
-      <c r="L17" s="14"/>
-    </row>
-    <row r="18" spans="1:12" s="11" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="34"/>
-      <c r="B18" s="31"/>
-      <c r="C18" s="28"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="9"/>
-      <c r="H18" s="9"/>
-      <c r="I18" s="9"/>
-      <c r="J18" s="9"/>
-      <c r="K18" s="10"/>
-      <c r="L18" s="13"/>
-    </row>
-    <row r="19" spans="1:12" s="7" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="33"/>
-      <c r="B19" s="30"/>
-      <c r="C19" s="27"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="5"/>
-      <c r="K19" s="6"/>
-      <c r="L19" s="14"/>
-    </row>
-    <row r="20" spans="1:12" s="11" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="34"/>
-      <c r="B20" s="31"/>
-      <c r="C20" s="28"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="9"/>
-      <c r="H20" s="9"/>
-      <c r="I20" s="9"/>
-      <c r="J20" s="9"/>
-      <c r="K20" s="10"/>
-      <c r="L20" s="13"/>
-    </row>
-    <row r="21" spans="1:12" s="7" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="33"/>
-      <c r="B21" s="30"/>
-      <c r="C21" s="27"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
-      <c r="J21" s="5"/>
-      <c r="K21" s="6"/>
-      <c r="L21" s="14"/>
-    </row>
-    <row r="22" spans="1:12" s="11" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="34"/>
-      <c r="B22" s="31"/>
-      <c r="C22" s="28"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
-      <c r="G22" s="9"/>
-      <c r="H22" s="9"/>
-      <c r="I22" s="9"/>
-      <c r="J22" s="9"/>
-      <c r="K22" s="10"/>
-      <c r="L22" s="13"/>
+      <c r="D4" s="29">
+        <v>0.02</v>
+      </c>
+      <c r="E4" s="30">
+        <v>1.7999999999999999E-2</v>
+      </c>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+      <c r="J4" s="30">
+        <v>0.157</v>
+      </c>
+      <c r="K4" s="30">
+        <v>0.01</v>
+      </c>
+      <c r="L4" s="30">
+        <v>11.728999999999999</v>
+      </c>
+      <c r="M4" s="30">
+        <v>0.14199999999999999</v>
+      </c>
+      <c r="N4" s="30">
+        <v>0.3755</v>
+      </c>
+      <c r="O4" s="31">
+        <v>0.1066</v>
+      </c>
+      <c r="P4" s="25" t="str">
+        <f t="shared" ref="P4:P22" si="0">TEXT(SUM(D4:O4)/1440,"hh:mm:ss")</f>
+        <v>00:12:33</v>
+      </c>
+      <c r="Q4" s="38" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" s="1" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="22" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="19">
+        <v>120</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="26">
+        <v>4.7E-2</v>
+      </c>
+      <c r="E5" s="27">
+        <v>9.9000000000000005E-2</v>
+      </c>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="27"/>
+      <c r="I5" s="27"/>
+      <c r="J5" s="27">
+        <v>1.0880000000000001</v>
+      </c>
+      <c r="K5" s="27">
+        <v>2E-3</v>
+      </c>
+      <c r="L5" s="27">
+        <v>33.747</v>
+      </c>
+      <c r="M5" s="27">
+        <v>0.439</v>
+      </c>
+      <c r="N5" s="27">
+        <v>0.82099999999999995</v>
+      </c>
+      <c r="O5" s="28">
+        <v>0.31648516666999998</v>
+      </c>
+      <c r="P5" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>00:36:34</v>
+      </c>
+      <c r="Q5" s="37" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" s="2" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="20">
+        <v>45</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="29">
+        <v>1.9E-2</v>
+      </c>
+      <c r="E6" s="30">
+        <v>2.3E-2</v>
+      </c>
+      <c r="F6" s="30"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="30"/>
+      <c r="J6" s="30">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="K6" s="30">
+        <v>1E-3</v>
+      </c>
+      <c r="L6" s="30">
+        <v>11.417999999999999</v>
+      </c>
+      <c r="M6" s="30">
+        <v>0.152</v>
+      </c>
+      <c r="N6" s="30">
+        <v>0.37730000000000002</v>
+      </c>
+      <c r="O6" s="31">
+        <v>6.8099999999999994E-2</v>
+      </c>
+      <c r="P6" s="25" t="str">
+        <f t="shared" si="0"/>
+        <v>00:12:25</v>
+      </c>
+      <c r="Q6" s="38" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" s="1" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="22"/>
+      <c r="B7" s="19"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="26"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="27"/>
+      <c r="I7" s="27"/>
+      <c r="J7" s="27"/>
+      <c r="K7" s="27"/>
+      <c r="L7" s="27"/>
+      <c r="M7" s="27"/>
+      <c r="N7" s="27"/>
+      <c r="O7" s="28"/>
+      <c r="P7" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>00:00:00</v>
+      </c>
+      <c r="Q7" s="37" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" s="2" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="23"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
+      <c r="J8" s="30"/>
+      <c r="K8" s="30"/>
+      <c r="L8" s="30"/>
+      <c r="M8" s="30"/>
+      <c r="N8" s="30"/>
+      <c r="O8" s="31"/>
+      <c r="P8" s="25" t="str">
+        <f t="shared" si="0"/>
+        <v>00:00:00</v>
+      </c>
+      <c r="Q8" s="38"/>
+    </row>
+    <row r="9" spans="1:17" s="1" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="22"/>
+      <c r="B9" s="19"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="26"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+      <c r="G9" s="27"/>
+      <c r="H9" s="27"/>
+      <c r="I9" s="27"/>
+      <c r="J9" s="27"/>
+      <c r="K9" s="27"/>
+      <c r="L9" s="27"/>
+      <c r="M9" s="27"/>
+      <c r="N9" s="27"/>
+      <c r="O9" s="28"/>
+      <c r="P9" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>00:00:00</v>
+      </c>
+      <c r="Q9" s="37"/>
+    </row>
+    <row r="10" spans="1:17" s="2" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="23"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="30"/>
+      <c r="J10" s="30"/>
+      <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
+      <c r="M10" s="30"/>
+      <c r="N10" s="30"/>
+      <c r="O10" s="31"/>
+      <c r="P10" s="25" t="str">
+        <f t="shared" si="0"/>
+        <v>00:00:00</v>
+      </c>
+      <c r="Q10" s="38"/>
+    </row>
+    <row r="11" spans="1:17" s="1" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="22"/>
+      <c r="B11" s="19"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="27"/>
+      <c r="I11" s="27"/>
+      <c r="J11" s="27"/>
+      <c r="K11" s="27"/>
+      <c r="L11" s="27"/>
+      <c r="M11" s="27"/>
+      <c r="N11" s="27"/>
+      <c r="O11" s="28"/>
+      <c r="P11" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>00:00:00</v>
+      </c>
+      <c r="Q11" s="37"/>
+    </row>
+    <row r="12" spans="1:17" s="2" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="23"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="29"/>
+      <c r="E12" s="30"/>
+      <c r="F12" s="30"/>
+      <c r="G12" s="30"/>
+      <c r="H12" s="30"/>
+      <c r="I12" s="30"/>
+      <c r="J12" s="30"/>
+      <c r="K12" s="30"/>
+      <c r="L12" s="30"/>
+      <c r="M12" s="30"/>
+      <c r="N12" s="30"/>
+      <c r="O12" s="31"/>
+      <c r="P12" s="25" t="str">
+        <f t="shared" si="0"/>
+        <v>00:00:00</v>
+      </c>
+      <c r="Q12" s="38"/>
+    </row>
+    <row r="13" spans="1:17" s="1" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="22"/>
+      <c r="B13" s="19"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="27"/>
+      <c r="F13" s="27"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="27"/>
+      <c r="I13" s="27"/>
+      <c r="J13" s="27"/>
+      <c r="K13" s="27"/>
+      <c r="L13" s="27"/>
+      <c r="M13" s="27"/>
+      <c r="N13" s="27"/>
+      <c r="O13" s="28"/>
+      <c r="P13" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>00:00:00</v>
+      </c>
+      <c r="Q13" s="37"/>
+    </row>
+    <row r="14" spans="1:17" s="2" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="23"/>
+      <c r="B14" s="20"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="30"/>
+      <c r="G14" s="30"/>
+      <c r="H14" s="30"/>
+      <c r="I14" s="30"/>
+      <c r="J14" s="30"/>
+      <c r="K14" s="30"/>
+      <c r="L14" s="30"/>
+      <c r="M14" s="30"/>
+      <c r="N14" s="30"/>
+      <c r="O14" s="31"/>
+      <c r="P14" s="25" t="str">
+        <f t="shared" si="0"/>
+        <v>00:00:00</v>
+      </c>
+      <c r="Q14" s="38"/>
+    </row>
+    <row r="15" spans="1:17" s="1" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="22"/>
+      <c r="B15" s="19"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="26"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="27"/>
+      <c r="J15" s="27"/>
+      <c r="K15" s="27"/>
+      <c r="L15" s="27"/>
+      <c r="M15" s="27"/>
+      <c r="N15" s="27"/>
+      <c r="O15" s="28"/>
+      <c r="P15" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>00:00:00</v>
+      </c>
+      <c r="Q15" s="37"/>
+    </row>
+    <row r="16" spans="1:17" s="2" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="23"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="30"/>
+      <c r="F16" s="30"/>
+      <c r="G16" s="30"/>
+      <c r="H16" s="30"/>
+      <c r="I16" s="30"/>
+      <c r="J16" s="30"/>
+      <c r="K16" s="30"/>
+      <c r="L16" s="30"/>
+      <c r="M16" s="30"/>
+      <c r="N16" s="30"/>
+      <c r="O16" s="31"/>
+      <c r="P16" s="25" t="str">
+        <f t="shared" si="0"/>
+        <v>00:00:00</v>
+      </c>
+      <c r="Q16" s="38"/>
+    </row>
+    <row r="17" spans="1:17" s="1" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="22"/>
+      <c r="B17" s="19"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="26"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="27"/>
+      <c r="H17" s="27"/>
+      <c r="I17" s="27"/>
+      <c r="J17" s="27"/>
+      <c r="K17" s="27"/>
+      <c r="L17" s="27"/>
+      <c r="M17" s="27"/>
+      <c r="N17" s="27"/>
+      <c r="O17" s="28"/>
+      <c r="P17" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>00:00:00</v>
+      </c>
+      <c r="Q17" s="37"/>
+    </row>
+    <row r="18" spans="1:17" s="2" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="23"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="30"/>
+      <c r="H18" s="30"/>
+      <c r="I18" s="30"/>
+      <c r="J18" s="30"/>
+      <c r="K18" s="30"/>
+      <c r="L18" s="30"/>
+      <c r="M18" s="30"/>
+      <c r="N18" s="30"/>
+      <c r="O18" s="31"/>
+      <c r="P18" s="25" t="str">
+        <f t="shared" si="0"/>
+        <v>00:00:00</v>
+      </c>
+      <c r="Q18" s="38"/>
+    </row>
+    <row r="19" spans="1:17" s="1" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="22"/>
+      <c r="B19" s="19"/>
+      <c r="C19" s="16"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="27"/>
+      <c r="H19" s="27"/>
+      <c r="I19" s="27"/>
+      <c r="J19" s="27"/>
+      <c r="K19" s="27"/>
+      <c r="L19" s="27"/>
+      <c r="M19" s="27"/>
+      <c r="N19" s="27"/>
+      <c r="O19" s="28"/>
+      <c r="P19" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>00:00:00</v>
+      </c>
+      <c r="Q19" s="37"/>
+    </row>
+    <row r="20" spans="1:17" s="2" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="23"/>
+      <c r="B20" s="20"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="30"/>
+      <c r="F20" s="30"/>
+      <c r="G20" s="30"/>
+      <c r="H20" s="30"/>
+      <c r="I20" s="30"/>
+      <c r="J20" s="30"/>
+      <c r="K20" s="30"/>
+      <c r="L20" s="30"/>
+      <c r="M20" s="30"/>
+      <c r="N20" s="30"/>
+      <c r="O20" s="31"/>
+      <c r="P20" s="25" t="str">
+        <f t="shared" si="0"/>
+        <v>00:00:00</v>
+      </c>
+      <c r="Q20" s="38"/>
+    </row>
+    <row r="21" spans="1:17" s="1" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="22"/>
+      <c r="B21" s="19"/>
+      <c r="C21" s="16"/>
+      <c r="D21" s="26"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="27"/>
+      <c r="H21" s="27"/>
+      <c r="I21" s="27"/>
+      <c r="J21" s="27"/>
+      <c r="K21" s="27"/>
+      <c r="L21" s="27"/>
+      <c r="M21" s="27"/>
+      <c r="N21" s="27"/>
+      <c r="O21" s="28"/>
+      <c r="P21" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>00:00:00</v>
+      </c>
+      <c r="Q21" s="37"/>
+    </row>
+    <row r="22" spans="1:17" s="2" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="23"/>
+      <c r="B22" s="20"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="30"/>
+      <c r="F22" s="30"/>
+      <c r="G22" s="30"/>
+      <c r="H22" s="30"/>
+      <c r="I22" s="30"/>
+      <c r="J22" s="30"/>
+      <c r="K22" s="30"/>
+      <c r="L22" s="30"/>
+      <c r="M22" s="30"/>
+      <c r="N22" s="30"/>
+      <c r="O22" s="31"/>
+      <c r="P22" s="25" t="str">
+        <f t="shared" si="0"/>
+        <v>00:00:00</v>
+      </c>
+      <c r="Q22" s="38"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="G1:K1"/>
-    <mergeCell ref="L1:L2"/>
+  <mergeCells count="9">
+    <mergeCell ref="K1:O1"/>
+    <mergeCell ref="P1:P2"/>
+    <mergeCell ref="E1:I1"/>
+    <mergeCell ref="Q1:Q2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="J1:J2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C78B30D-2D9D-440A-9BF4-0390A3946410}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>